<commit_message>
Add Excel learning files
</commit_message>
<xml_diff>
--- a/introducion.xlsx
+++ b/introducion.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kirti Gupta\Desktop\EXCEL LEARNINGS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{242E6145-0A1E-4561-AAAD-FD73F3D8CC10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE366DA-D53B-44CD-B4AF-042F90BB07E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{65952268-C3B1-4105-BD6A-EF210D4F0D64}"/>
   </bookViews>
@@ -264,7 +264,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="25" x14ac:knownFonts="1">
     <font>
@@ -554,12 +554,6 @@
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -573,7 +567,7 @@
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -582,12 +576,18 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -916,19 +916,19 @@
     <col min="6" max="6" width="26.88671875" style="5" customWidth="1"/>
     <col min="7" max="7" width="24.77734375" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" customWidth="1"/>
-    <col min="9" max="9" width="15.6640625" style="19" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" style="17" customWidth="1"/>
     <col min="10" max="10" width="15.6640625" customWidth="1"/>
     <col min="11" max="11" width="31.88671875" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:13" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
     </row>
     <row r="3" spans="3:13" ht="27.6" x14ac:dyDescent="0.65">
       <c r="C3" s="8" t="s">
@@ -946,7 +946,7 @@
       <c r="G3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="19">
+      <c r="I3" s="17">
         <v>89</v>
       </c>
       <c r="J3">
@@ -963,7 +963,7 @@
       </c>
     </row>
     <row r="4" spans="3:13" x14ac:dyDescent="0.45">
-      <c r="I4" s="19">
+      <c r="I4" s="17">
         <v>65</v>
       </c>
       <c r="J4">
@@ -980,7 +980,7 @@
       </c>
     </row>
     <row r="5" spans="3:13" x14ac:dyDescent="0.45">
-      <c r="I5" s="19">
+      <c r="I5" s="17">
         <v>78</v>
       </c>
       <c r="J5">
@@ -997,14 +997,14 @@
       </c>
     </row>
     <row r="6" spans="3:13" ht="25.2" x14ac:dyDescent="0.5">
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="I6" s="19">
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="I6" s="17">
         <v>89</v>
       </c>
       <c r="J6">
@@ -1021,7 +1021,7 @@
       </c>
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.45">
-      <c r="I7" s="19">
+      <c r="I7" s="17">
         <v>1000</v>
       </c>
       <c r="J7">
@@ -1055,7 +1055,7 @@
       </c>
     </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.45">
-      <c r="I10" s="19">
+      <c r="I10" s="17">
         <v>8</v>
       </c>
       <c r="K10" s="11">
@@ -1064,7 +1064,7 @@
     </row>
     <row r="11" spans="3:13" x14ac:dyDescent="0.45">
       <c r="E11" s="1"/>
-      <c r="I11" s="19">
+      <c r="I11" s="17">
         <v>78</v>
       </c>
       <c r="K11" s="11">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" s="14"/>
-      <c r="G26" s="20" t="s">
+      <c r="G26" s="18" t="s">
         <v>63</v>
       </c>
       <c r="H26" s="2"/>
@@ -1210,7 +1210,7 @@
       <c r="H27" t="s">
         <v>37</v>
       </c>
-      <c r="I27" s="19" t="s">
+      <c r="I27" s="17" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       <c r="H28" t="s">
         <v>40</v>
       </c>
-      <c r="I28" s="19" t="s">
+      <c r="I28" s="17" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       <c r="H29" t="s">
         <v>50</v>
       </c>
-      <c r="I29" s="19" t="s">
+      <c r="I29" s="17" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       <c r="H30" t="s">
         <v>51</v>
       </c>
-      <c r="I30" s="19" t="s">
+      <c r="I30" s="17" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1290,7 +1290,7 @@
       <c r="H31" t="s">
         <v>52</v>
       </c>
-      <c r="I31" s="19" t="s">
+      <c r="I31" s="17" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       <c r="H32" t="s">
         <v>53</v>
       </c>
-      <c r="I32" s="19" t="s">
+      <c r="I32" s="17" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       <c r="H33" t="s">
         <v>54</v>
       </c>
-      <c r="I33" s="19" t="s">
+      <c r="I33" s="17" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       <c r="H34" t="s">
         <v>55</v>
       </c>
-      <c r="I34" s="19" t="s">
+      <c r="I34" s="17" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       <c r="H35" t="s">
         <v>56</v>
       </c>
-      <c r="I35" s="19" t="s">
+      <c r="I35" s="17" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1390,25 +1390,25 @@
       <c r="H36" t="s">
         <v>57</v>
       </c>
-      <c r="I36" s="19" t="s">
+      <c r="I36" s="17" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="39" spans="4:9" ht="29.4" x14ac:dyDescent="0.65">
-      <c r="D39" s="22" t="s">
+      <c r="D39" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="E39" s="21"/>
-      <c r="F39" s="21"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
     </row>
     <row r="40" spans="4:9" ht="21" x14ac:dyDescent="0.4">
-      <c r="D40" s="23" t="s">
+      <c r="D40" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="E40" s="23" t="s">
+      <c r="E40" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F40" s="21" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
         <v>79</v>
       </c>
       <c r="F45" s="5">
-        <f t="shared" ref="F42:F46" si="0">D45+E45</f>
+        <f t="shared" ref="F45:F46" si="0">D45+E45</f>
         <v>202</v>
       </c>
     </row>
@@ -1485,20 +1485,20 @@
       </c>
     </row>
     <row r="49" spans="4:6" ht="28.2" x14ac:dyDescent="0.5">
-      <c r="D49" s="27" t="s">
+      <c r="D49" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="E49" s="28"/>
-      <c r="F49" s="28"/>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
     </row>
     <row r="50" spans="4:6" ht="21" x14ac:dyDescent="0.4">
-      <c r="D50" s="23" t="s">
+      <c r="D50" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="E50" s="23" t="s">
+      <c r="E50" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="F50" s="23" t="s">
+      <c r="F50" s="21" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1506,10 +1506,10 @@
       <c r="D51" t="s">
         <v>39</v>
       </c>
-      <c r="E51" s="24">
+      <c r="E51" s="22">
         <v>400000</v>
       </c>
-      <c r="F51" s="29">
+      <c r="F51" s="27">
         <f>E51+(E51*$E$61)</f>
         <v>480000</v>
       </c>
@@ -1518,10 +1518,10 @@
       <c r="D52" t="s">
         <v>42</v>
       </c>
-      <c r="E52" s="24">
+      <c r="E52" s="22">
         <v>500001</v>
       </c>
-      <c r="F52" s="29">
+      <c r="F52" s="27">
         <f>E52+(E52*$E$61)</f>
         <v>600001.19999999995</v>
       </c>
@@ -1530,11 +1530,11 @@
       <c r="D53" t="s">
         <v>43</v>
       </c>
-      <c r="E53" s="24">
+      <c r="E53" s="22">
         <v>600002</v>
       </c>
-      <c r="F53" s="29">
-        <f t="shared" ref="F52:F59" si="1">E53+(E53*$E$61)</f>
+      <c r="F53" s="27">
+        <f t="shared" ref="F53:F59" si="1">E53+(E53*$E$61)</f>
         <v>720002.4</v>
       </c>
     </row>
@@ -1542,10 +1542,10 @@
       <c r="D54" t="s">
         <v>44</v>
       </c>
-      <c r="E54" s="24">
+      <c r="E54" s="22">
         <v>900003</v>
       </c>
-      <c r="F54" s="29">
+      <c r="F54" s="27">
         <f>E54+(E54*$E$61)</f>
         <v>1080003.6000000001</v>
       </c>
@@ -1554,10 +1554,10 @@
       <c r="D55" t="s">
         <v>45</v>
       </c>
-      <c r="E55" s="24">
+      <c r="E55" s="22">
         <v>300004</v>
       </c>
-      <c r="F55" s="29">
+      <c r="F55" s="27">
         <f>E55+(E55*$E$61)</f>
         <v>360004.8</v>
       </c>
@@ -1566,10 +1566,10 @@
       <c r="D56" t="s">
         <v>46</v>
       </c>
-      <c r="E56" s="24">
+      <c r="E56" s="22">
         <v>700005</v>
       </c>
-      <c r="F56" s="29">
+      <c r="F56" s="27">
         <f>E56+(E56*$E$61)</f>
         <v>840006</v>
       </c>
@@ -1578,10 +1578,10 @@
       <c r="D57" t="s">
         <v>47</v>
       </c>
-      <c r="E57" s="24">
+      <c r="E57" s="22">
         <v>700006</v>
       </c>
-      <c r="F57" s="29">
+      <c r="F57" s="27">
         <f t="shared" si="1"/>
         <v>840007.2</v>
       </c>
@@ -1590,10 +1590,10 @@
       <c r="D58" t="s">
         <v>48</v>
       </c>
-      <c r="E58" s="24">
+      <c r="E58" s="22">
         <v>900007</v>
       </c>
-      <c r="F58" s="29">
+      <c r="F58" s="27">
         <f>E58+(E58*$E$61)</f>
         <v>1080008.3999999999</v>
       </c>
@@ -1602,41 +1602,41 @@
       <c r="D59" t="s">
         <v>49</v>
       </c>
-      <c r="E59" s="24">
+      <c r="E59" s="22">
         <v>800008</v>
       </c>
-      <c r="F59" s="29">
+      <c r="F59" s="27">
         <f t="shared" si="1"/>
         <v>960009.6</v>
       </c>
     </row>
     <row r="61" spans="4:6" ht="25.2" x14ac:dyDescent="0.6">
-      <c r="D61" s="25" t="s">
+      <c r="D61" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="E61" s="26">
+      <c r="E61" s="24">
         <v>0.2</v>
       </c>
     </row>
     <row r="65" spans="4:7" ht="27.6" x14ac:dyDescent="0.45">
-      <c r="D65" s="30" t="s">
+      <c r="D65" s="28" t="s">
         <v>70</v>
       </c>
-      <c r="E65" s="30"/>
-      <c r="F65" s="30"/>
-      <c r="G65" s="30"/>
+      <c r="E65" s="28"/>
+      <c r="F65" s="28"/>
+      <c r="G65" s="28"/>
     </row>
     <row r="66" spans="4:7" ht="21" x14ac:dyDescent="0.4">
-      <c r="D66" s="23" t="s">
+      <c r="D66" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="E66" s="23" t="s">
+      <c r="E66" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="F66" s="23" t="s">
+      <c r="F66" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="G66" s="23" t="s">
+      <c r="G66" s="21" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1644,10 +1644,10 @@
       <c r="D67" t="s">
         <v>39</v>
       </c>
-      <c r="E67" s="24">
+      <c r="E67" s="22">
         <v>400000</v>
       </c>
-      <c r="F67" s="29">
+      <c r="F67" s="27">
         <f>E67+(E67*E77)</f>
         <v>480000</v>
       </c>
@@ -1656,7 +1656,7 @@
       <c r="D68" t="s">
         <v>42</v>
       </c>
-      <c r="E68" s="24">
+      <c r="E68" s="22">
         <v>500001</v>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       <c r="D69" t="s">
         <v>43</v>
       </c>
-      <c r="E69" s="24">
+      <c r="E69" s="22">
         <v>600002</v>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       <c r="D70" t="s">
         <v>44</v>
       </c>
-      <c r="E70" s="24">
+      <c r="E70" s="22">
         <v>900003</v>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       <c r="D71" t="s">
         <v>45</v>
       </c>
-      <c r="E71" s="24">
+      <c r="E71" s="22">
         <v>300004</v>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       <c r="D72" t="s">
         <v>46</v>
       </c>
-      <c r="E72" s="24">
+      <c r="E72" s="22">
         <v>700005</v>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       <c r="D73" t="s">
         <v>47</v>
       </c>
-      <c r="E73" s="24">
+      <c r="E73" s="22">
         <v>700006</v>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       <c r="D74" t="s">
         <v>48</v>
       </c>
-      <c r="E74" s="24">
+      <c r="E74" s="22">
         <v>900007</v>
       </c>
     </row>
@@ -1712,23 +1712,23 @@
       <c r="D75" t="s">
         <v>49</v>
       </c>
-      <c r="E75" s="24">
+      <c r="E75" s="22">
         <v>800008</v>
       </c>
     </row>
     <row r="77" spans="4:7" ht="25.2" x14ac:dyDescent="0.6">
-      <c r="D77" s="25" t="s">
+      <c r="D77" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="E77" s="26">
+      <c r="E77" s="24">
         <v>0.2</v>
       </c>
     </row>
     <row r="78" spans="4:7" ht="32.4" x14ac:dyDescent="0.7">
-      <c r="D78" s="31" t="s">
+      <c r="D78" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="E78" s="32">
+      <c r="E78" s="30">
         <v>0.05</v>
       </c>
     </row>

</xml_diff>